<commit_message>
Add megger model, W/m and PE1402 failed-megger deficiency for 10-01
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WvWi9nyBzSNkvytisZiLo5
</commit_message>
<xml_diff>
--- a/10-01_GIM_GONCHO/E&I-QAQC-Deficiency-Tracker- UPDATED.xlsx
+++ b/10-01_GIM_GONCHO/E&I-QAQC-Deficiency-Tracker- UPDATED.xlsx
@@ -16409,18 +16409,60 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="B256" s="47"/>
-      <c r="C256" s="39"/>
-      <c r="D256" s="39"/>
-      <c r="E256" s="39"/>
-      <c r="F256" s="39"/>
-      <c r="G256" s="20"/>
-      <c r="H256" s="39"/>
-      <c r="I256" s="44"/>
-      <c r="J256" s="39"/>
-      <c r="K256" s="39"/>
+      <c r="B256" s="47">
+        <v>46246</v>
+      </c>
+      <c r="C256" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29103-WPM-102</t>
+        </is>
+      </c>
+      <c r="D256" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K1B-600V-EHT</t>
+        </is>
+      </c>
+      <c r="E256" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrical</t>
+        </is>
+      </c>
+      <c r="F256" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29103-ET-PE1402-1-1</t>
+        </is>
+      </c>
+      <c r="G256" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YCQE-EHT-003 (2026-08-12); YCQE-EHT-QF-13.1</t>
+        </is>
+      </c>
+      <c r="H256" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testing</t>
+        </is>
+      </c>
+      <c r="I256" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pre-insulation megger FAILED (0.0 MOhm @ 500 VDC); trace not released for insulation. Temp tags - EHT and RTD need SS tags.</t>
+        </is>
+      </c>
+      <c r="J256" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="K256" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Construction</t>
+        </is>
+      </c>
       <c r="L256" s="26"/>
-      <c r="M256" s="39"/>
+      <c r="M256" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
       <c r="N256" s="26"/>
       <c r="O256" s="20"/>
       <c r="P256" s="26"/>
@@ -16433,7 +16475,11 @@
         <v/>
       </c>
       <c r="S256" s="17"/>
-      <c r="T256" s="32"/>
+      <c r="T256" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From EHT-003 by Robert Dixon 2026/08/12. MI continuity 44.9 Ohm. Panel 29103-HTP-003 CB-33.</t>
+        </is>
+      </c>
     </row>
     <row r="257" spans="1:20">
       <c r="A257" s="23" t="str">

</xml_diff>

<commit_message>
Set System by pattern: RTDs = process service, power kits = HTP panel
RTD test records use the line service (PE/P = PRODUCED EMULSION, etc.)
with the HTP panel moved to the controller box. Drain Tank power kit
reports get 29152-HTP-001 from 29152-65H-102-01. Punchlist 1 tracker
tags expanded per 29151-65H-102-01 (Drain Tank 1, DT-29151).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WvWi9nyBzSNkvytisZiLo5
</commit_message>
<xml_diff>
--- a/10-01_GIM_GONCHO/E&I-QAQC-Deficiency-Tracker- UPDATED.xlsx
+++ b/10-01_GIM_GONCHO/E&I-QAQC-Deficiency-Tracker- UPDATED.xlsx
@@ -14412,12 +14412,12 @@
       </c>
       <c r="C230" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D230" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E230" s="39" t="inlineStr">
@@ -14427,7 +14427,7 @@
       </c>
       <c r="F230" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">TANK1-1-PWK</t>
+          <t xml:space="preserve">TANK1-1-PWK-1</t>
         </is>
       </c>
       <c r="G230" s="20" t="inlineStr">
@@ -14475,7 +14475,7 @@
       <c r="S230" s="17"/>
       <c r="T230" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist category C. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist category C. Tank 1 tag (not in cable schedule); -1 suffix added to match TANK2 format.</t>
         </is>
       </c>
     </row>
@@ -14489,12 +14489,12 @@
       </c>
       <c r="C231" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D231" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E231" s="39" t="inlineStr">
@@ -14504,7 +14504,7 @@
       </c>
       <c r="F231" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ETHC-4102-PWK</t>
+          <t xml:space="preserve">29151-ET-HC4102-1-PWK-1</t>
         </is>
       </c>
       <c r="G231" s="20" t="inlineStr">
@@ -14552,7 +14552,7 @@
       <c r="S231" s="17"/>
       <c r="T231" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
         </is>
       </c>
     </row>
@@ -14566,12 +14566,12 @@
       </c>
       <c r="C232" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D232" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E232" s="39" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F232" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ETFG-4102-PWK</t>
+          <t xml:space="preserve">29151-ET-FG4102-1-PWK-1</t>
         </is>
       </c>
       <c r="G232" s="20" t="inlineStr">
@@ -14629,7 +14629,7 @@
       <c r="S232" s="17"/>
       <c r="T232" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
         </is>
       </c>
     </row>
@@ -14643,12 +14643,12 @@
       </c>
       <c r="C233" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D233" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E233" s="39" t="inlineStr">
@@ -14658,7 +14658,7 @@
       </c>
       <c r="F233" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ETDR-4100-PWK</t>
+          <t xml:space="preserve">29151-ET-DR4100-1-PWK-1</t>
         </is>
       </c>
       <c r="G233" s="20" t="inlineStr">
@@ -14706,7 +14706,7 @@
       <c r="S233" s="17"/>
       <c r="T233" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
         </is>
       </c>
     </row>
@@ -14720,12 +14720,12 @@
       </c>
       <c r="C234" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D234" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E234" s="39" t="inlineStr">
@@ -14735,7 +14735,7 @@
       </c>
       <c r="F234" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ETHC-5008-PWK</t>
+          <t xml:space="preserve">29203-ET-HC5008-1-PWK-1</t>
         </is>
       </c>
       <c r="G234" s="20" t="inlineStr">
@@ -14783,7 +14783,7 @@
       <c r="S234" s="17"/>
       <c r="T234" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
         </is>
       </c>
     </row>
@@ -14797,12 +14797,12 @@
       </c>
       <c r="C235" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D235" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E235" s="39" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F235" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ETPE-5002-PWK / ETPE-5002-2-R1</t>
+          <t xml:space="preserve">29203-ET-PE5002-2-PWK-1 / 29203-ET-PE5002-2-R-1</t>
         </is>
       </c>
       <c r="G235" s="20" t="inlineStr">
@@ -14860,7 +14860,7 @@
       <c r="S235" s="17"/>
       <c r="T235" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
         </is>
       </c>
     </row>
@@ -14874,12 +14874,12 @@
       </c>
       <c r="C236" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D236" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E236" s="39" t="inlineStr">
@@ -14889,7 +14889,7 @@
       </c>
       <c r="F236" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">TANK1-5-PWK</t>
+          <t xml:space="preserve">TANK1-5-PWK-1</t>
         </is>
       </c>
       <c r="G236" s="20" t="inlineStr">
@@ -14937,7 +14937,7 @@
       <c r="S236" s="17"/>
       <c r="T236" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Tank 1 tag (not in cable schedule); -1 suffix added to match TANK2 format.</t>
         </is>
       </c>
     </row>
@@ -14951,12 +14951,12 @@
       </c>
       <c r="C237" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D237" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E237" s="39" t="inlineStr">
@@ -14966,7 +14966,7 @@
       </c>
       <c r="F237" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ETMT-0002-PWK</t>
+          <t xml:space="preserve">29151-ET-MT0002-1-PWK-3</t>
         </is>
       </c>
       <c r="G237" s="20" t="inlineStr">
@@ -15014,7 +15014,7 @@
       <c r="S237" s="17"/>
       <c r="T237" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
         </is>
       </c>
     </row>
@@ -15028,12 +15028,12 @@
       </c>
       <c r="C238" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D238" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E238" s="39" t="inlineStr">
@@ -15043,7 +15043,7 @@
       </c>
       <c r="F238" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ETPG-4100-PWK</t>
+          <t xml:space="preserve">29151-ET-PG4100-1-PWK-1</t>
         </is>
       </c>
       <c r="G238" s="20" t="inlineStr">
@@ -15091,7 +15091,7 @@
       <c r="S238" s="17"/>
       <c r="T238" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
         </is>
       </c>
     </row>
@@ -15105,12 +15105,12 @@
       </c>
       <c r="C239" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1</t>
+          <t xml:space="preserve">Drain Tank 1 (29151)</t>
         </is>
       </c>
       <c r="D239" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple</t>
+          <t xml:space="preserve">DT-29151</t>
         </is>
       </c>
       <c r="E239" s="39" t="inlineStr">
@@ -15168,7 +15168,7 @@
       <c r="S239" s="17"/>
       <c r="T239" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tag as written on punchlist.</t>
+          <t xml:space="preserve">Punched by Murtesa / Liam. Tank 1 tag (not in cable schedule); as written.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Name reports by tag only; keep scan remarks verbatim; drop notes files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WvWi9nyBzSNkvytisZiLo5
</commit_message>
<xml_diff>
--- a/10-01_GIM_GONCHO/E&I-QAQC-Deficiency-Tracker- UPDATED.xlsx
+++ b/10-01_GIM_GONCHO/E&I-QAQC-Deficiency-Tracker- UPDATED.xlsx
@@ -14412,7 +14412,7 @@
       </c>
       <c r="C230" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D230" s="39" t="inlineStr">
@@ -14430,11 +14430,7 @@
           <t xml:space="preserve">TANK1-1-PWK-1</t>
         </is>
       </c>
-      <c r="G230" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G230" s="20"/>
       <c r="H230" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -14473,11 +14469,7 @@
         <v/>
       </c>
       <c r="S230" s="17"/>
-      <c r="T230" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist category C. Tank 1 tag (not in cable schedule); -1 suffix added to match TANK2 format.</t>
-        </is>
-      </c>
+      <c r="T230" s="32"/>
     </row>
     <row r="231" spans="1:20">
       <c r="A231" s="23" t="str">
@@ -14489,7 +14481,7 @@
       </c>
       <c r="C231" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D231" s="39" t="inlineStr">
@@ -14507,11 +14499,7 @@
           <t xml:space="preserve">29151-ET-HC4102-1-PWK-1</t>
         </is>
       </c>
-      <c r="G231" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G231" s="20"/>
       <c r="H231" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -14550,11 +14538,7 @@
         <v/>
       </c>
       <c r="S231" s="17"/>
-      <c r="T231" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
-        </is>
-      </c>
+      <c r="T231" s="32"/>
     </row>
     <row r="232" spans="1:20">
       <c r="A232" s="23" t="str">
@@ -14566,7 +14550,7 @@
       </c>
       <c r="C232" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D232" s="39" t="inlineStr">
@@ -14584,11 +14568,7 @@
           <t xml:space="preserve">29151-ET-FG4102-1-PWK-1</t>
         </is>
       </c>
-      <c r="G232" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G232" s="20"/>
       <c r="H232" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -14627,11 +14607,7 @@
         <v/>
       </c>
       <c r="S232" s="17"/>
-      <c r="T232" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
-        </is>
-      </c>
+      <c r="T232" s="32"/>
     </row>
     <row r="233" spans="1:20">
       <c r="A233" s="23" t="str">
@@ -14643,7 +14619,7 @@
       </c>
       <c r="C233" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D233" s="39" t="inlineStr">
@@ -14661,11 +14637,7 @@
           <t xml:space="preserve">29151-ET-DR4100-1-PWK-1</t>
         </is>
       </c>
-      <c r="G233" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G233" s="20"/>
       <c r="H233" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -14704,11 +14676,7 @@
         <v/>
       </c>
       <c r="S233" s="17"/>
-      <c r="T233" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
-        </is>
-      </c>
+      <c r="T233" s="32"/>
     </row>
     <row r="234" spans="1:20">
       <c r="A234" s="23" t="str">
@@ -14720,7 +14688,7 @@
       </c>
       <c r="C234" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D234" s="39" t="inlineStr">
@@ -14738,11 +14706,7 @@
           <t xml:space="preserve">29203-ET-HC5008-1-PWK-1</t>
         </is>
       </c>
-      <c r="G234" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G234" s="20"/>
       <c r="H234" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -14781,11 +14745,7 @@
         <v/>
       </c>
       <c r="S234" s="17"/>
-      <c r="T234" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
-        </is>
-      </c>
+      <c r="T234" s="32"/>
     </row>
     <row r="235" spans="1:20">
       <c r="A235" s="23" t="str">
@@ -14797,7 +14757,7 @@
       </c>
       <c r="C235" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D235" s="39" t="inlineStr">
@@ -14815,11 +14775,7 @@
           <t xml:space="preserve">29203-ET-PE5002-2-PWK-1 / 29203-ET-PE5002-2-R-1</t>
         </is>
       </c>
-      <c r="G235" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G235" s="20"/>
       <c r="H235" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -14858,11 +14814,7 @@
         <v/>
       </c>
       <c r="S235" s="17"/>
-      <c r="T235" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
-        </is>
-      </c>
+      <c r="T235" s="32"/>
     </row>
     <row r="236" spans="1:20">
       <c r="A236" s="23" t="str">
@@ -14874,7 +14826,7 @@
       </c>
       <c r="C236" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D236" s="39" t="inlineStr">
@@ -14892,11 +14844,7 @@
           <t xml:space="preserve">TANK1-5-PWK-1</t>
         </is>
       </c>
-      <c r="G236" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G236" s="20"/>
       <c r="H236" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -14935,11 +14883,7 @@
         <v/>
       </c>
       <c r="S236" s="17"/>
-      <c r="T236" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tank 1 tag (not in cable schedule); -1 suffix added to match TANK2 format.</t>
-        </is>
-      </c>
+      <c r="T236" s="32"/>
     </row>
     <row r="237" spans="1:20">
       <c r="A237" s="23" t="str">
@@ -14951,7 +14895,7 @@
       </c>
       <c r="C237" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D237" s="39" t="inlineStr">
@@ -14969,11 +14913,7 @@
           <t xml:space="preserve">29151-ET-MT0002-1-PWK-3</t>
         </is>
       </c>
-      <c r="G237" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G237" s="20"/>
       <c r="H237" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15012,11 +14952,7 @@
         <v/>
       </c>
       <c r="S237" s="17"/>
-      <c r="T237" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
-        </is>
-      </c>
+      <c r="T237" s="32"/>
     </row>
     <row r="238" spans="1:20">
       <c r="A238" s="23" t="str">
@@ -15028,7 +14964,7 @@
       </c>
       <c r="C238" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D238" s="39" t="inlineStr">
@@ -15046,11 +14982,7 @@
           <t xml:space="preserve">29151-ET-PG4100-1-PWK-1</t>
         </is>
       </c>
-      <c r="G238" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G238" s="20"/>
       <c r="H238" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15089,11 +15021,7 @@
         <v/>
       </c>
       <c r="S238" s="17"/>
-      <c r="T238" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Punchlist tag expanded per 29151-65H-102-01 (29151-HTP-001).</t>
-        </is>
-      </c>
+      <c r="T238" s="32"/>
     </row>
     <row r="239" spans="1:20">
       <c r="A239" s="23" t="str">
@@ -15105,7 +15033,7 @@
       </c>
       <c r="C239" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drain Tank 1 (29151)</t>
+          <t xml:space="preserve">Drain Tank 1</t>
         </is>
       </c>
       <c r="D239" s="39" t="inlineStr">
@@ -15123,11 +15051,7 @@
           <t xml:space="preserve">TANK1-3-R-1</t>
         </is>
       </c>
-      <c r="G239" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 (2026-09-27)</t>
-        </is>
-      </c>
+      <c r="G239" s="20"/>
       <c r="H239" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15166,11 +15090,7 @@
         <v/>
       </c>
       <c r="S239" s="17"/>
-      <c r="T239" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Tank 1 tag (not in cable schedule); as written.</t>
-        </is>
-      </c>
+      <c r="T239" s="32"/>
     </row>
     <row r="240" spans="1:20">
       <c r="A240" s="23" t="str">
@@ -15200,11 +15120,7 @@
           <t xml:space="preserve">29103-ET-PE1102-1-PWK-1</t>
         </is>
       </c>
-      <c r="G240" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29); YCQE-E&amp;I-113</t>
-        </is>
-      </c>
+      <c r="G240" s="20"/>
       <c r="H240" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15243,11 +15159,7 @@
         <v/>
       </c>
       <c r="S240" s="17"/>
-      <c r="T240" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Combined: punchlist item + small power ITR remarks.</t>
-        </is>
-      </c>
+      <c r="T240" s="32"/>
     </row>
     <row r="241" spans="1:20">
       <c r="A241" s="23" t="str">
@@ -15277,11 +15189,7 @@
           <t xml:space="preserve">29103-ET-PE1201-1-PWK-1</t>
         </is>
       </c>
-      <c r="G241" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29); YCQE-E&amp;I-113</t>
-        </is>
-      </c>
+      <c r="G241" s="20"/>
       <c r="H241" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15320,11 +15228,7 @@
         <v/>
       </c>
       <c r="S241" s="17"/>
-      <c r="T241" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Combined: punchlist item + small power ITR remarks.</t>
-        </is>
-      </c>
+      <c r="T241" s="32"/>
     </row>
     <row r="242" spans="1:20">
       <c r="A242" s="23" t="str">
@@ -15354,11 +15258,7 @@
           <t xml:space="preserve">29103-ET-P1204-2-PWK-1</t>
         </is>
       </c>
-      <c r="G242" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29); YCQE-E&amp;I-113</t>
-        </is>
-      </c>
+      <c r="G242" s="20"/>
       <c r="H242" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15397,11 +15297,7 @@
         <v/>
       </c>
       <c r="S242" s="17"/>
-      <c r="T242" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Combined: punchlist item + small power ITR remarks.</t>
-        </is>
-      </c>
+      <c r="T242" s="32"/>
     </row>
     <row r="243" spans="1:20">
       <c r="A243" s="23" t="str">
@@ -15431,11 +15327,7 @@
           <t xml:space="preserve">29103-ET-PG1201-2-PWK-1</t>
         </is>
       </c>
-      <c r="G243" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="G243" s="20"/>
       <c r="H243" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15474,11 +15366,7 @@
         <v/>
       </c>
       <c r="S243" s="17"/>
-      <c r="T243" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam.</t>
-        </is>
-      </c>
+      <c r="T243" s="32"/>
     </row>
     <row r="244" spans="1:20">
       <c r="A244" s="23" t="str">
@@ -15508,11 +15396,7 @@
           <t xml:space="preserve">29103-ET-PE1802-1-PWK-1</t>
         </is>
       </c>
-      <c r="G244" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29); YCQE-E&amp;I-113</t>
-        </is>
-      </c>
+      <c r="G244" s="20"/>
       <c r="H244" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15551,11 +15435,7 @@
         <v/>
       </c>
       <c r="S244" s="17"/>
-      <c r="T244" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Combined: punchlist item + small power ITR remarks.</t>
-        </is>
-      </c>
+      <c r="T244" s="32"/>
     </row>
     <row r="245" spans="1:20">
       <c r="A245" s="23" t="str">
@@ -15585,11 +15465,7 @@
           <t xml:space="preserve">29103-ET-ST1103-1-PWK-1</t>
         </is>
       </c>
-      <c r="G245" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="G245" s="20"/>
       <c r="H245" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15628,11 +15504,7 @@
         <v/>
       </c>
       <c r="S245" s="17"/>
-      <c r="T245" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam.</t>
-        </is>
-      </c>
+      <c r="T245" s="32"/>
     </row>
     <row r="246" spans="1:20">
       <c r="A246" s="23" t="str">
@@ -15662,11 +15534,7 @@
           <t xml:space="preserve">29103-ET-FG1203-1-PWK-1</t>
         </is>
       </c>
-      <c r="G246" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="G246" s="20"/>
       <c r="H246" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15705,11 +15573,7 @@
         <v/>
       </c>
       <c r="S246" s="17"/>
-      <c r="T246" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam.</t>
-        </is>
-      </c>
+      <c r="T246" s="32"/>
     </row>
     <row r="247" spans="1:20">
       <c r="A247" s="23" t="str">
@@ -15739,11 +15603,7 @@
           <t xml:space="preserve">29103-ET-PG1101-2-PWK-1</t>
         </is>
       </c>
-      <c r="G247" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="G247" s="20"/>
       <c r="H247" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15782,11 +15642,7 @@
         <v/>
       </c>
       <c r="S247" s="17"/>
-      <c r="T247" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam.</t>
-        </is>
-      </c>
+      <c r="T247" s="32"/>
     </row>
     <row r="248" spans="1:20">
       <c r="A248" s="23" t="str">
@@ -15816,11 +15672,7 @@
           <t xml:space="preserve">29103-ET-FG1105-1-PWK-1</t>
         </is>
       </c>
-      <c r="G248" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="G248" s="20"/>
       <c r="H248" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15859,11 +15711,7 @@
         <v/>
       </c>
       <c r="S248" s="17"/>
-      <c r="T248" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam.</t>
-        </is>
-      </c>
+      <c r="T248" s="32"/>
     </row>
     <row r="249" spans="1:20">
       <c r="A249" s="23" t="str">
@@ -15893,11 +15741,7 @@
           <t xml:space="preserve">29103-ET-PE1101-2-PWK-1</t>
         </is>
       </c>
-      <c r="G249" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="G249" s="20"/>
       <c r="H249" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -15936,11 +15780,7 @@
         <v/>
       </c>
       <c r="S249" s="17"/>
-      <c r="T249" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam.</t>
-        </is>
-      </c>
+      <c r="T249" s="32"/>
     </row>
     <row r="250" spans="1:20">
       <c r="A250" s="23" t="str">
@@ -15970,11 +15810,7 @@
           <t xml:space="preserve">29103-ET-PE1101-1-PWK-1</t>
         </is>
       </c>
-      <c r="G250" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="G250" s="20"/>
       <c r="H250" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -16013,11 +15849,7 @@
         <v/>
       </c>
       <c r="S250" s="17"/>
-      <c r="T250" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Note: small power ITR for this cable (Sept 28) shows all items initialed with no remarks - verify.</t>
-        </is>
-      </c>
+      <c r="T250" s="32"/>
     </row>
     <row r="251" spans="1:20">
       <c r="A251" s="23" t="str">
@@ -16047,11 +15879,7 @@
           <t xml:space="preserve">29103-ET-P1201-1-PWK-1</t>
         </is>
       </c>
-      <c r="G251" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29); YCQE-E&amp;I-113</t>
-        </is>
-      </c>
+      <c r="G251" s="20"/>
       <c r="H251" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -16090,11 +15918,7 @@
         <v/>
       </c>
       <c r="S251" s="17"/>
-      <c r="T251" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Combined: punchlist item + small power ITR remarks.</t>
-        </is>
-      </c>
+      <c r="T251" s="32"/>
     </row>
     <row r="252" spans="1:20">
       <c r="A252" s="23" t="str">
@@ -16124,11 +15948,7 @@
           <t xml:space="preserve">29103-ET-ST1001-1-PWK-1</t>
         </is>
       </c>
-      <c r="G252" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29)</t>
-        </is>
-      </c>
+      <c r="G252" s="20"/>
       <c r="H252" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -16167,11 +15987,7 @@
         <v/>
       </c>
       <c r="S252" s="17"/>
-      <c r="T252" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam.</t>
-        </is>
-      </c>
+      <c r="T252" s="32"/>
     </row>
     <row r="253" spans="1:20">
       <c r="A253" s="23" t="str">
@@ -16201,11 +16017,7 @@
           <t xml:space="preserve">29103-ET-P1104-2-PWK-1</t>
         </is>
       </c>
-      <c r="G253" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29); YCQE-E&amp;I-113</t>
-        </is>
-      </c>
+      <c r="G253" s="20"/>
       <c r="H253" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -16244,11 +16056,7 @@
         <v/>
       </c>
       <c r="S253" s="17"/>
-      <c r="T253" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Combined with small power ITR (scan read PE1104-2; cable schedule 29103-65H-102-01 confirms P1104-2).</t>
-        </is>
-      </c>
+      <c r="T253" s="32"/>
     </row>
     <row r="254" spans="1:20">
       <c r="A254" s="23" t="str">
@@ -16278,11 +16086,7 @@
           <t xml:space="preserve">29103-ET-PG1101-1-PWK-1</t>
         </is>
       </c>
-      <c r="G254" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-PS-048 Internal (2026-09-29); YCQE-E&amp;I-113</t>
-        </is>
-      </c>
+      <c r="G254" s="20"/>
       <c r="H254" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -16321,11 +16125,7 @@
         <v/>
       </c>
       <c r="S254" s="17"/>
-      <c r="T254" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punched by Murtesa / Liam. Combined: punchlist item + small power ITR remarks.</t>
-        </is>
-      </c>
+      <c r="T254" s="32"/>
     </row>
     <row r="255" spans="1:20">
       <c r="A255" s="23" t="str">
@@ -16355,11 +16155,7 @@
           <t xml:space="preserve">29103-ET-P1101-1-PWK-1</t>
         </is>
       </c>
-      <c r="G255" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-E&amp;I-113</t>
-        </is>
-      </c>
+      <c r="G255" s="20"/>
       <c r="H255" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Installation</t>
@@ -16398,11 +16194,7 @@
         <v/>
       </c>
       <c r="S255" s="17"/>
-      <c r="T255" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From small power ITR remarks (Sept 29); not on punchlist.</t>
-        </is>
-      </c>
+      <c r="T255" s="32"/>
     </row>
     <row r="256" spans="1:20">
       <c r="A256" s="23" t="str">
@@ -16432,11 +16224,7 @@
           <t xml:space="preserve">29103-ET-PE1402-1-1</t>
         </is>
       </c>
-      <c r="G256" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YCQE-EHT-003 (2026-08-12); YCQE-EHT-QF-13.1</t>
-        </is>
-      </c>
+      <c r="G256" s="20"/>
       <c r="H256" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Testing</t>
@@ -16444,7 +16232,7 @@
       </c>
       <c r="I256" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-insulation megger FAILED (0.0 MOhm @ 500 VDC); trace not released for insulation. Temp tags - EHT and RTD need SS tags.</t>
+          <t xml:space="preserve">Failed megger 0.0 MΩ. Temp tags, EHT and RTD need SS tags.</t>
         </is>
       </c>
       <c r="J256" s="39" t="inlineStr">
@@ -16475,11 +16263,7 @@
         <v/>
       </c>
       <c r="S256" s="17"/>
-      <c r="T256" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From EHT-003 by Robert Dixon 2026/08/12. MI continuity 44.9 Ohm. Panel 29103-HTP-003 CB-33.</t>
-        </is>
-      </c>
+      <c r="T256" s="32"/>
     </row>
     <row r="257" spans="1:20">
       <c r="A257" s="23" t="str">

</xml_diff>